<commit_message>
Tested montecarlo with goal of least emissions
</commit_message>
<xml_diff>
--- a/Versionen/emissionen_als_neg_sp/game_data.xlsx
+++ b/Versionen/emissionen_als_neg_sp/game_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schneids\code\KlimSta-Brettspiel\Versionen\emissionen_als_neg_sp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Documents\_Privat\Coding\KlimSta\Versionen\emissionen_als_neg_sp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ED0F8CF-AA8B-4675-B890-3014791B3F09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C53287AB-75AE-4624-B2C6-22B209AB57FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-18120" windowWidth="29040" windowHeight="17520" tabRatio="721" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="721" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Massnahmenkarten Spielwerte" sheetId="1" r:id="rId1"/>
@@ -73,9 +73,9 @@
   <commentList>
     <comment ref="C1" authorId="0" shapeId="0" xr:uid="{884F3275-8B47-4A24-9A63-26455AFB7D59}">
       <text>
-        <t>[Kommentarthread]
-Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
-Kommentar:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     KgCO2/m²a</t>
       </text>
     </comment>
@@ -92,18 +92,18 @@
   <commentList>
     <comment ref="C2" authorId="0" shapeId="0" xr:uid="{EF592111-A8C2-4853-9B03-5FD652A65E13}">
       <text>
-        <t xml:space="preserve">[Kommentarthread]
-Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
-Kommentar:
+        <t xml:space="preserve">[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     €/m²
 </t>
       </text>
     </comment>
     <comment ref="H2" authorId="1" shapeId="0" xr:uid="{42E090DF-C6E0-4ACF-94D0-539FD66BF793}">
       <text>
-        <t>[Kommentarthread]
-Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
-Kommentar:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     Geld token</t>
       </text>
     </comment>
@@ -1791,7 +1791,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="140">
+  <cellXfs count="138">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -2185,65 +2185,21 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="1" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="78">
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFB4E5A2"/>
-          <bgColor rgb="FFB4E5A2"/>
+          <fgColor rgb="FFB7E1CD"/>
+          <bgColor rgb="FFB7E1CD"/>
         </patternFill>
       </fill>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color rgb="FFB4E5A2"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFB4E5A2"/>
-        </right>
-        <top style="thin">
-          <color rgb="FFB4E5A2"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FFB4E5A2"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
@@ -2274,123 +2230,6 @@
         <scheme val="minor"/>
       </font>
       <numFmt numFmtId="164" formatCode="0.0"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="164" formatCode="0.0"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB7E1CD"/>
-          <bgColor rgb="FFB7E1CD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-      </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -2447,6 +2286,44 @@
         <name val="Arial"/>
         <scheme val="minor"/>
       </font>
+      <numFmt numFmtId="164" formatCode="0.0"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+      </font>
       <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -2466,10 +2343,23 @@
         <name val="Arial"/>
         <scheme val="minor"/>
       </font>
+      <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
       <font>
@@ -2487,6 +2377,7 @@
         <name val="Arial"/>
         <scheme val="minor"/>
       </font>
+      <numFmt numFmtId="1" formatCode="0"/>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -2506,142 +2397,6 @@
         <scheme val="minor"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="7" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Arial"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Roboto"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB4E5A2"/>
-          <bgColor rgb="FFB4E5A2"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center" textRotation="90" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <font>
@@ -2835,6 +2590,245 @@
         <name val="Arial"/>
         <scheme val="minor"/>
       </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Roboto"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB4E5A2"/>
+          <bgColor rgb="FFB4E5A2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="90" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB4E5A2"/>
+          <bgColor rgb="FFB4E5A2"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFB4E5A2"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFB4E5A2"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFB4E5A2"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFB4E5A2"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="7" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Arial"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="5" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -3237,16 +3231,16 @@
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Heizsystem"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Kosten"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="BauEmissionen"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="SofortCO2" dataDxfId="34">
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="SofortCO2" dataDxfId="43">
       <calculatedColumnFormula>Table1[[#This Row],[REAL Sofort CO2]]/kgemission_per_sp</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Strombedarf" dataDxfId="33">
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Strombedarf" dataDxfId="42">
       <calculatedColumnFormula>Table1[[#This Row],[REAL Strombedarf]]/real_zu_spiel_strombedarf</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Stromproduktion" dataDxfId="1">
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Stromproduktion" dataDxfId="41">
       <calculatedColumnFormula>Table1[[#This Row],[REAL Stromproduktion]]/real_zu_spiel_stromproduktion</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Stromspeicher" dataDxfId="0">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Stromspeicher" dataDxfId="40">
       <calculatedColumnFormula>Table1[[#This Row],[REAL Stromspeicher]]/real_zu_spiel_stromspeicher</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Wärmeschutz"/>
@@ -3254,8 +3248,8 @@
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Zufriedenheit"/>
     <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="SofortBudget"/>
     <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="REAL Kosten"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="REAL BauEmissionen" dataDxfId="2"/>
-    <tableColumn id="25" xr3:uid="{8B6CFA43-B9CB-4808-B66A-C728842AC947}" name="REAL Sofort CO2" dataDxfId="32"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="REAL BauEmissionen" dataDxfId="39"/>
+    <tableColumn id="25" xr3:uid="{8B6CFA43-B9CB-4808-B66A-C728842AC947}" name="REAL Sofort CO2" dataDxfId="38"/>
     <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="REAL Strombedarf"/>
     <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="REAL Stromproduktion"/>
     <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="REAL Stromspeicher"/>
@@ -3289,8 +3283,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table3" displayName="Table3" ref="A1:E34">
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Wert"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Real" dataDxfId="31"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Spiel" dataDxfId="30"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Real" dataDxfId="45"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Spiel" dataDxfId="44"/>
     <tableColumn id="5" xr3:uid="{16BD6806-29CB-4A81-B6F6-E74363828D03}" name="Skalierung real &gt; spiel"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Einheit"/>
   </tableColumns>
@@ -3323,19 +3317,19 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="Table6" displayName="Table6" ref="A1:L11">
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="WS"/>
-    <tableColumn id="12" xr3:uid="{EB8234D1-70DE-48AE-82B3-197397D4EA50}" name="HWB" dataDxfId="29"/>
-    <tableColumn id="7" xr3:uid="{382715DF-E649-4C68-8229-17F79CFD05E9}" name="Gas Real" dataDxfId="28"/>
-    <tableColumn id="8" xr3:uid="{9D3BFB1F-D194-4CFF-801A-646B03B69223}" name="Biomasse Real" dataDxfId="27"/>
-    <tableColumn id="9" xr3:uid="{92D64809-6003-4492-A647-B5959B9DDB64}" name="Fernwärme Real" dataDxfId="26"/>
-    <tableColumn id="10" xr3:uid="{08723E33-0A65-4BFC-9E7A-BA30B56D6C93}" name="Grünes Gas Real" dataDxfId="25"/>
-    <tableColumn id="11" xr3:uid="{308CC45B-DB70-43B9-B4BC-DFAA9033E01B}" name="Wärmepumpe Real" dataDxfId="24"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Gas" dataDxfId="23">
+    <tableColumn id="12" xr3:uid="{EB8234D1-70DE-48AE-82B3-197397D4EA50}" name="HWB" dataDxfId="37"/>
+    <tableColumn id="7" xr3:uid="{382715DF-E649-4C68-8229-17F79CFD05E9}" name="Gas Real" dataDxfId="36"/>
+    <tableColumn id="8" xr3:uid="{9D3BFB1F-D194-4CFF-801A-646B03B69223}" name="Biomasse Real" dataDxfId="35"/>
+    <tableColumn id="9" xr3:uid="{92D64809-6003-4492-A647-B5959B9DDB64}" name="Fernwärme Real" dataDxfId="34"/>
+    <tableColumn id="10" xr3:uid="{08723E33-0A65-4BFC-9E7A-BA30B56D6C93}" name="Grünes Gas Real" dataDxfId="33"/>
+    <tableColumn id="11" xr3:uid="{308CC45B-DB70-43B9-B4BC-DFAA9033E01B}" name="Wärmepumpe Real" dataDxfId="32"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Gas" dataDxfId="31">
       <calculatedColumnFormula>Table6[[#This Row],[Gas Real]]*years_per_round</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="Biomasse">
       <calculatedColumnFormula>Table6[[#This Row],[Biomasse Real]]*years_per_round</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="Fernwärme" dataDxfId="22">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="Fernwärme" dataDxfId="30">
       <calculatedColumnFormula>Table6[[#This Row],[Fernwärme Real]]*years_per_round</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="Grünes Gas">
@@ -3353,35 +3347,35 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="Table6_2" displayName="Table6_2" ref="A1:L11">
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="WS"/>
-    <tableColumn id="12" xr3:uid="{0F5289D2-6D79-4CC0-B64B-353B2E52E442}" name="HWB" dataDxfId="45"/>
-    <tableColumn id="7" xr3:uid="{7EE7A865-A9C3-4293-93B4-6A7F6B0D0739}" name="Gas Real" dataDxfId="44">
+    <tableColumn id="12" xr3:uid="{0F5289D2-6D79-4CC0-B64B-353B2E52E442}" name="HWB" dataDxfId="29"/>
+    <tableColumn id="7" xr3:uid="{7EE7A865-A9C3-4293-93B4-6A7F6B0D0739}" name="Gas Real" dataDxfId="28">
       <calculatedColumnFormula>Table6_2[[#This Row],[HWB]]*'Mapping RealwerteSpielwerte'!$B$23</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{B9056603-4120-4751-8FD5-39C0A331CEB9}" name="Biomasse Real" dataDxfId="43">
+    <tableColumn id="8" xr3:uid="{B9056603-4120-4751-8FD5-39C0A331CEB9}" name="Biomasse Real" dataDxfId="27">
       <calculatedColumnFormula>Table6_2[[#This Row],[HWB]]*'Mapping RealwerteSpielwerte'!$B$24</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{775B0FD7-CE79-4EF3-8952-C905936C6A82}" name="Fernwärme Real" dataDxfId="42">
+    <tableColumn id="9" xr3:uid="{775B0FD7-CE79-4EF3-8952-C905936C6A82}" name="Fernwärme Real" dataDxfId="26">
       <calculatedColumnFormula>Table6_2[[#This Row],[HWB]]*'Mapping RealwerteSpielwerte'!$B$25</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{600AB853-60A0-47F9-B6B9-14F74CC0E0AE}" name="Grünes Gas Real" dataDxfId="41">
+    <tableColumn id="10" xr3:uid="{600AB853-60A0-47F9-B6B9-14F74CC0E0AE}" name="Grünes Gas Real" dataDxfId="25">
       <calculatedColumnFormula>Table6_2[[#This Row],[HWB]]*'Mapping RealwerteSpielwerte'!$B$26</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{1611B9F2-405C-4348-B6D7-02BE82C080AD}" name="Wärmepumpe Real" dataDxfId="40">
+    <tableColumn id="11" xr3:uid="{1611B9F2-405C-4348-B6D7-02BE82C080AD}" name="Wärmepumpe Real" dataDxfId="24">
       <calculatedColumnFormula>0</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="Gas" dataDxfId="39">
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="Gas" dataDxfId="23">
       <calculatedColumnFormula>-Table6_2[[#This Row],[Gas Real]]*'Mapping RealwerteSpielwerte'!$C$23+heizkosten_baseline</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="Biomasse" dataDxfId="38">
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="Biomasse" dataDxfId="22">
       <calculatedColumnFormula>-Table6_2[[#This Row],[Biomasse Real]]*'Mapping RealwerteSpielwerte'!$C$24+heizkosten_baseline</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="Fernwärme" dataDxfId="37">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="Fernwärme" dataDxfId="21">
       <calculatedColumnFormula>-Table6_2[[#This Row],[Fernwärme Real]]*'Mapping RealwerteSpielwerte'!$C$25+heizkosten_baseline</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" name="Grünes Gas" dataDxfId="36">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" name="Grünes Gas" dataDxfId="20">
       <calculatedColumnFormula>-Table6_2[[#This Row],[Grünes Gas Real]]*'Mapping RealwerteSpielwerte'!$C$26+heizkosten_baseline</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="Wärmepumpe" dataDxfId="35">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="Wärmepumpe" dataDxfId="19">
       <calculatedColumnFormula>-Table6_2[[#This Row],[Wärmepumpe Real]]*'Mapping RealwerteSpielwerte'!$C$27+heizkosten_baseline</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3424,37 +3418,37 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF07000000}" name="Table8" displayName="Table8" ref="A1:L37">
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="Netzbezug"/>
-    <tableColumn id="7" xr3:uid="{FA3BADB2-767D-406F-AE0E-3FD85C94E47C}" name="Netzbezug Real" dataDxfId="21">
+    <tableColumn id="7" xr3:uid="{FA3BADB2-767D-406F-AE0E-3FD85C94E47C}" name="Netzbezug Real" dataDxfId="11">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug]]*real_zu_spiel_netzbezug</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="12" xr3:uid="{7CF654A3-746E-45BB-8FE8-D85A1A2F26B3}" name="Kosten Real" dataDxfId="10">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug Real]]*'Mapping RealwerteSpielwerte'!$B$27</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Budget" dataDxfId="8">
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Budget" dataDxfId="9">
       <calculatedColumnFormula>-Table8[[#This Row],[Kosten Real]]*'Mapping RealwerteSpielwerte'!$C$27</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{CF2B80D5-564A-4F28-96D5-E05D40FB1362}" name="Emissionen Runde 1 Real" dataDxfId="9">
+    <tableColumn id="8" xr3:uid="{CF2B80D5-564A-4F28-96D5-E05D40FB1362}" name="Emissionen Runde 1 Real" dataDxfId="8">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{DDA1FEAD-C691-4D07-9868-BA59E3083198}" name="Emissionen Runde 2 Real" dataDxfId="20">
+    <tableColumn id="9" xr3:uid="{DDA1FEAD-C691-4D07-9868-BA59E3083198}" name="Emissionen Runde 2 Real" dataDxfId="7">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{FA64A352-3640-4484-B5E7-A06D893CF066}" name="Emissionen Runde 3 Real" dataDxfId="19">
+    <tableColumn id="10" xr3:uid="{FA64A352-3640-4484-B5E7-A06D893CF066}" name="Emissionen Runde 3 Real" dataDxfId="6">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{D2D0C651-2DB4-4AE8-8AC2-5459168B14AC}" name="Emissionen Runde 4 Real" dataDxfId="7">
+    <tableColumn id="11" xr3:uid="{D2D0C651-2DB4-4AE8-8AC2-5459168B14AC}" name="Emissionen Runde 4 Real" dataDxfId="5">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="SP Runde 1" dataDxfId="6">
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="SP Runde 1" dataDxfId="4">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="SP Runde 2" dataDxfId="5">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0700-000004000000}" name="SP Runde 2" dataDxfId="3">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0700-000005000000}" name="SP Runde 3" dataDxfId="4">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0700-000005000000}" name="SP Runde 3" dataDxfId="2">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0700-000006000000}" name="SP Runde 4" dataDxfId="3">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0700-000006000000}" name="SP Runde 4" dataDxfId="1">
       <calculatedColumnFormula>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3720,7 +3714,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:Y1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.453125" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -3895,7 +3889,7 @@
       <c r="M3" s="23"/>
       <c r="N3" s="24"/>
       <c r="O3" s="25"/>
-      <c r="P3" s="139">
+      <c r="P3" s="16">
         <v>-5</v>
       </c>
       <c r="Q3" s="37"/>
@@ -32663,7 +32657,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="O1:V1 O2:O100 Q73:V100">
-    <cfRule type="expression" dxfId="11" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>"T"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -32686,7 +32680,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:V993"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.453125" customWidth="1"/>
     <col min="2" max="4" width="35.1796875" customWidth="1"/>
@@ -57365,7 +57359,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:M35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.54296875" customWidth="1"/>
     <col min="5" max="5" width="21.7265625" customWidth="1"/>
@@ -57726,7 +57720,7 @@
       <c r="A23" t="s">
         <v>331</v>
       </c>
-      <c r="B23" s="137">
+      <c r="B23" s="120">
         <v>0.1</v>
       </c>
       <c r="C23" s="126">
@@ -57744,7 +57738,7 @@
       <c r="A24" t="s">
         <v>332</v>
       </c>
-      <c r="B24" s="137">
+      <c r="B24" s="120">
         <v>0.08</v>
       </c>
       <c r="C24" s="126">
@@ -57762,7 +57756,7 @@
       <c r="A25" t="s">
         <v>333</v>
       </c>
-      <c r="B25" s="137">
+      <c r="B25" s="120">
         <v>0.2</v>
       </c>
       <c r="C25" s="126">
@@ -57780,7 +57774,7 @@
       <c r="A26" t="s">
         <v>334</v>
       </c>
-      <c r="B26" s="137">
+      <c r="B26" s="120">
         <v>0.5</v>
       </c>
       <c r="C26" s="126">
@@ -57798,7 +57792,7 @@
       <c r="A27" t="s">
         <v>335</v>
       </c>
-      <c r="B27" s="137">
+      <c r="B27" s="120">
         <v>0.15</v>
       </c>
       <c r="C27" s="126">
@@ -57825,7 +57819,7 @@
       <c r="A29" t="s">
         <v>339</v>
       </c>
-      <c r="B29" s="137">
+      <c r="B29" s="120">
         <v>1</v>
       </c>
       <c r="C29" s="126">
@@ -57840,7 +57834,7 @@
       <c r="A30" t="s">
         <v>340</v>
       </c>
-      <c r="B30" s="137">
+      <c r="B30" s="120">
         <v>2</v>
       </c>
       <c r="C30" s="126">
@@ -57855,7 +57849,7 @@
       <c r="A31" t="s">
         <v>341</v>
       </c>
-      <c r="B31" s="137">
+      <c r="B31" s="120">
         <v>2.5</v>
       </c>
       <c r="C31" s="126">
@@ -57870,7 +57864,7 @@
       <c r="A32" t="s">
         <v>342</v>
       </c>
-      <c r="B32" s="137">
+      <c r="B32" s="120">
         <v>3.3330000000000002</v>
       </c>
       <c r="C32" s="126">
@@ -57885,7 +57879,7 @@
       <c r="A33" t="s">
         <v>343</v>
       </c>
-      <c r="B33" s="137">
+      <c r="B33" s="120">
         <v>4.5454499999999998</v>
       </c>
       <c r="C33" s="126">
@@ -57900,7 +57894,7 @@
       <c r="A34" t="s">
         <v>344</v>
       </c>
-      <c r="B34" s="137">
+      <c r="B34" s="120">
         <v>6.66</v>
       </c>
       <c r="C34" s="126">
@@ -57934,7 +57928,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:M6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.54296875" customWidth="1"/>
     <col min="2" max="2" width="17.26953125" customWidth="1"/>
@@ -58202,7 +58196,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:L11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="9" max="9" width="12.81640625" customWidth="1"/>
     <col min="10" max="10" width="13.81640625" customWidth="1"/>
@@ -58699,7 +58693,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:L11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="9" max="9" width="12.81640625" customWidth="1"/>
     <col min="10" max="10" width="13.81640625" customWidth="1"/>
@@ -59270,7 +59264,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:H25"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="8" width="13.1796875" customWidth="1"/>
   </cols>
@@ -59713,7 +59707,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:L37"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.7265625" customWidth="1"/>
     <col min="10" max="13" width="14" customWidth="1"/>
@@ -59789,19 +59783,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>0</v>
       </c>
-      <c r="I2" s="138">
+      <c r="I2" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>0</v>
       </c>
-      <c r="J2" s="138">
+      <c r="J2" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>0</v>
       </c>
-      <c r="K2" s="138">
+      <c r="K2" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>0</v>
       </c>
-      <c r="L2" s="138">
+      <c r="L2" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>0</v>
       </c>
@@ -59838,19 +59832,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>0.375</v>
       </c>
-      <c r="I3" s="138">
+      <c r="I3" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>2.5</v>
       </c>
-      <c r="J3" s="138">
+      <c r="J3" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>1.25</v>
       </c>
-      <c r="K3" s="138">
+      <c r="K3" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>0.75</v>
       </c>
-      <c r="L3" s="138">
+      <c r="L3" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>0.375</v>
       </c>
@@ -59887,19 +59881,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>0.75</v>
       </c>
-      <c r="I4" s="138">
+      <c r="I4" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>5</v>
       </c>
-      <c r="J4" s="138">
+      <c r="J4" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>2.5</v>
       </c>
-      <c r="K4" s="138">
+      <c r="K4" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>1.5</v>
       </c>
-      <c r="L4" s="138">
+      <c r="L4" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>0.75</v>
       </c>
@@ -59936,19 +59930,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>1.125</v>
       </c>
-      <c r="I5" s="138">
+      <c r="I5" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>7.5</v>
       </c>
-      <c r="J5" s="138">
+      <c r="J5" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>3.75</v>
       </c>
-      <c r="K5" s="138">
+      <c r="K5" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>2.25</v>
       </c>
-      <c r="L5" s="138">
+      <c r="L5" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>1.125</v>
       </c>
@@ -59985,19 +59979,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>1.5</v>
       </c>
-      <c r="I6" s="138">
+      <c r="I6" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>10</v>
       </c>
-      <c r="J6" s="138">
+      <c r="J6" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>5</v>
       </c>
-      <c r="K6" s="138">
+      <c r="K6" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>3</v>
       </c>
-      <c r="L6" s="138">
+      <c r="L6" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>1.5</v>
       </c>
@@ -60034,19 +60028,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>1.875</v>
       </c>
-      <c r="I7" s="138">
+      <c r="I7" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>12.5</v>
       </c>
-      <c r="J7" s="138">
+      <c r="J7" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>6.25</v>
       </c>
-      <c r="K7" s="138">
+      <c r="K7" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>3.75</v>
       </c>
-      <c r="L7" s="138">
+      <c r="L7" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>1.875</v>
       </c>
@@ -60083,19 +60077,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>2.25</v>
       </c>
-      <c r="I8" s="138">
+      <c r="I8" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>15</v>
       </c>
-      <c r="J8" s="138">
+      <c r="J8" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>7.5</v>
       </c>
-      <c r="K8" s="138">
+      <c r="K8" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>4.5</v>
       </c>
-      <c r="L8" s="138">
+      <c r="L8" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>2.25</v>
       </c>
@@ -60132,19 +60126,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>2.625</v>
       </c>
-      <c r="I9" s="138">
+      <c r="I9" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>17.5</v>
       </c>
-      <c r="J9" s="138">
+      <c r="J9" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>8.75</v>
       </c>
-      <c r="K9" s="138">
+      <c r="K9" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>5.25</v>
       </c>
-      <c r="L9" s="138">
+      <c r="L9" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>2.625</v>
       </c>
@@ -60181,19 +60175,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>3</v>
       </c>
-      <c r="I10" s="138">
+      <c r="I10" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>20</v>
       </c>
-      <c r="J10" s="138">
+      <c r="J10" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>10</v>
       </c>
-      <c r="K10" s="138">
+      <c r="K10" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>6</v>
       </c>
-      <c r="L10" s="138">
+      <c r="L10" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>3</v>
       </c>
@@ -60230,19 +60224,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>3.3749999999999996</v>
       </c>
-      <c r="I11" s="138">
+      <c r="I11" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>22.5</v>
       </c>
-      <c r="J11" s="138">
+      <c r="J11" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>11.25</v>
       </c>
-      <c r="K11" s="138">
+      <c r="K11" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>6.7499999999999991</v>
       </c>
-      <c r="L11" s="138">
+      <c r="L11" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>3.3749999999999996</v>
       </c>
@@ -60279,19 +60273,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>3.75</v>
       </c>
-      <c r="I12" s="138">
+      <c r="I12" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>25</v>
       </c>
-      <c r="J12" s="138">
+      <c r="J12" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>12.5</v>
       </c>
-      <c r="K12" s="138">
+      <c r="K12" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>7.5</v>
       </c>
-      <c r="L12" s="138">
+      <c r="L12" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>3.75</v>
       </c>
@@ -60328,19 +60322,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>4.125</v>
       </c>
-      <c r="I13" s="138">
+      <c r="I13" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>27.5</v>
       </c>
-      <c r="J13" s="138">
+      <c r="J13" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>13.75</v>
       </c>
-      <c r="K13" s="138">
+      <c r="K13" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>8.25</v>
       </c>
-      <c r="L13" s="138">
+      <c r="L13" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>4.125</v>
       </c>
@@ -60377,19 +60371,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>4.5</v>
       </c>
-      <c r="I14" s="138">
+      <c r="I14" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>30</v>
       </c>
-      <c r="J14" s="138">
+      <c r="J14" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>15</v>
       </c>
-      <c r="K14" s="138">
+      <c r="K14" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>9</v>
       </c>
-      <c r="L14" s="138">
+      <c r="L14" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>4.5</v>
       </c>
@@ -60426,19 +60420,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>4.875</v>
       </c>
-      <c r="I15" s="138">
+      <c r="I15" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>32.5</v>
       </c>
-      <c r="J15" s="138">
+      <c r="J15" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>16.25</v>
       </c>
-      <c r="K15" s="138">
+      <c r="K15" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>9.75</v>
       </c>
-      <c r="L15" s="138">
+      <c r="L15" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>4.875</v>
       </c>
@@ -60475,19 +60469,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>5.25</v>
       </c>
-      <c r="I16" s="138">
+      <c r="I16" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>35</v>
       </c>
-      <c r="J16" s="138">
+      <c r="J16" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>17.5</v>
       </c>
-      <c r="K16" s="138">
+      <c r="K16" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>10.5</v>
       </c>
-      <c r="L16" s="138">
+      <c r="L16" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>5.25</v>
       </c>
@@ -60524,19 +60518,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>5.625</v>
       </c>
-      <c r="I17" s="138">
+      <c r="I17" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>37.5</v>
       </c>
-      <c r="J17" s="138">
+      <c r="J17" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>18.75</v>
       </c>
-      <c r="K17" s="138">
+      <c r="K17" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>11.25</v>
       </c>
-      <c r="L17" s="138">
+      <c r="L17" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>5.625</v>
       </c>
@@ -60573,19 +60567,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>6</v>
       </c>
-      <c r="I18" s="138">
+      <c r="I18" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>40</v>
       </c>
-      <c r="J18" s="138">
+      <c r="J18" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>20</v>
       </c>
-      <c r="K18" s="138">
+      <c r="K18" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>12</v>
       </c>
-      <c r="L18" s="138">
+      <c r="L18" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>6</v>
       </c>
@@ -60622,19 +60616,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>6.375</v>
       </c>
-      <c r="I19" s="138">
+      <c r="I19" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>42.5</v>
       </c>
-      <c r="J19" s="138">
+      <c r="J19" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>21.25</v>
       </c>
-      <c r="K19" s="138">
+      <c r="K19" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>12.75</v>
       </c>
-      <c r="L19" s="138">
+      <c r="L19" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>6.375</v>
       </c>
@@ -60671,19 +60665,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>6.7499999999999991</v>
       </c>
-      <c r="I20" s="138">
+      <c r="I20" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>45</v>
       </c>
-      <c r="J20" s="138">
+      <c r="J20" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>22.5</v>
       </c>
-      <c r="K20" s="138">
+      <c r="K20" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>13.499999999999998</v>
       </c>
-      <c r="L20" s="138">
+      <c r="L20" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>6.7499999999999991</v>
       </c>
@@ -60720,19 +60714,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>7.125</v>
       </c>
-      <c r="I21" s="138">
+      <c r="I21" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>47.5</v>
       </c>
-      <c r="J21" s="138">
+      <c r="J21" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>23.75</v>
       </c>
-      <c r="K21" s="138">
+      <c r="K21" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>14.25</v>
       </c>
-      <c r="L21" s="138">
+      <c r="L21" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>7.125</v>
       </c>
@@ -60769,19 +60763,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>7.5</v>
       </c>
-      <c r="I22" s="138">
+      <c r="I22" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>50</v>
       </c>
-      <c r="J22" s="138">
+      <c r="J22" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>25</v>
       </c>
-      <c r="K22" s="138">
+      <c r="K22" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>15</v>
       </c>
-      <c r="L22" s="138">
+      <c r="L22" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>7.5</v>
       </c>
@@ -60818,19 +60812,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>7.875</v>
       </c>
-      <c r="I23" s="138">
+      <c r="I23" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>52.5</v>
       </c>
-      <c r="J23" s="138">
+      <c r="J23" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>26.25</v>
       </c>
-      <c r="K23" s="138">
+      <c r="K23" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>15.75</v>
       </c>
-      <c r="L23" s="138">
+      <c r="L23" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>7.875</v>
       </c>
@@ -60867,19 +60861,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>8.25</v>
       </c>
-      <c r="I24" s="138">
+      <c r="I24" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>55</v>
       </c>
-      <c r="J24" s="138">
+      <c r="J24" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>27.5</v>
       </c>
-      <c r="K24" s="138">
+      <c r="K24" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>16.5</v>
       </c>
-      <c r="L24" s="138">
+      <c r="L24" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>8.25</v>
       </c>
@@ -60916,19 +60910,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>8.625</v>
       </c>
-      <c r="I25" s="138">
+      <c r="I25" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>57.5</v>
       </c>
-      <c r="J25" s="138">
+      <c r="J25" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>28.75</v>
       </c>
-      <c r="K25" s="138">
+      <c r="K25" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>17.25</v>
       </c>
-      <c r="L25" s="138">
+      <c r="L25" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>8.625</v>
       </c>
@@ -60965,19 +60959,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>9</v>
       </c>
-      <c r="I26" s="138">
+      <c r="I26" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>60</v>
       </c>
-      <c r="J26" s="138">
+      <c r="J26" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>30</v>
       </c>
-      <c r="K26" s="138">
+      <c r="K26" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>18</v>
       </c>
-      <c r="L26" s="138">
+      <c r="L26" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>9</v>
       </c>
@@ -61014,19 +61008,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>9.375</v>
       </c>
-      <c r="I27" s="138">
+      <c r="I27" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>62.5</v>
       </c>
-      <c r="J27" s="138">
+      <c r="J27" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>31.25</v>
       </c>
-      <c r="K27" s="138">
+      <c r="K27" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>18.75</v>
       </c>
-      <c r="L27" s="138">
+      <c r="L27" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>9.375</v>
       </c>
@@ -61063,19 +61057,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>9.75</v>
       </c>
-      <c r="I28" s="138">
+      <c r="I28" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>65</v>
       </c>
-      <c r="J28" s="138">
+      <c r="J28" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>32.5</v>
       </c>
-      <c r="K28" s="138">
+      <c r="K28" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>19.5</v>
       </c>
-      <c r="L28" s="138">
+      <c r="L28" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>9.75</v>
       </c>
@@ -61112,19 +61106,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>10.125</v>
       </c>
-      <c r="I29" s="138">
+      <c r="I29" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>67.5</v>
       </c>
-      <c r="J29" s="138">
+      <c r="J29" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>33.75</v>
       </c>
-      <c r="K29" s="138">
+      <c r="K29" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>20.25</v>
       </c>
-      <c r="L29" s="138">
+      <c r="L29" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>10.125</v>
       </c>
@@ -61161,19 +61155,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>10.5</v>
       </c>
-      <c r="I30" s="138">
+      <c r="I30" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>70</v>
       </c>
-      <c r="J30" s="138">
+      <c r="J30" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>35</v>
       </c>
-      <c r="K30" s="138">
+      <c r="K30" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>21</v>
       </c>
-      <c r="L30" s="138">
+      <c r="L30" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>10.5</v>
       </c>
@@ -61210,19 +61204,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>10.875</v>
       </c>
-      <c r="I31" s="138">
+      <c r="I31" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>72.5</v>
       </c>
-      <c r="J31" s="138">
+      <c r="J31" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>36.25</v>
       </c>
-      <c r="K31" s="138">
+      <c r="K31" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>21.75</v>
       </c>
-      <c r="L31" s="138">
+      <c r="L31" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>10.875</v>
       </c>
@@ -61259,19 +61253,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>11.25</v>
       </c>
-      <c r="I32" s="138">
+      <c r="I32" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>75</v>
       </c>
-      <c r="J32" s="138">
+      <c r="J32" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>37.5</v>
       </c>
-      <c r="K32" s="138">
+      <c r="K32" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>22.5</v>
       </c>
-      <c r="L32" s="138">
+      <c r="L32" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>11.25</v>
       </c>
@@ -61308,19 +61302,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>11.624999999999998</v>
       </c>
-      <c r="I33" s="138">
+      <c r="I33" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>77.5</v>
       </c>
-      <c r="J33" s="138">
+      <c r="J33" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>38.75</v>
       </c>
-      <c r="K33" s="138">
+      <c r="K33" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>23.249999999999996</v>
       </c>
-      <c r="L33" s="138">
+      <c r="L33" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>11.624999999999998</v>
       </c>
@@ -61357,19 +61351,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>12</v>
       </c>
-      <c r="I34" s="138">
+      <c r="I34" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>80</v>
       </c>
-      <c r="J34" s="138">
+      <c r="J34" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>40</v>
       </c>
-      <c r="K34" s="138">
+      <c r="K34" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>24</v>
       </c>
-      <c r="L34" s="138">
+      <c r="L34" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>12</v>
       </c>
@@ -61406,19 +61400,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>12.375</v>
       </c>
-      <c r="I35" s="138">
+      <c r="I35" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>82.5</v>
       </c>
-      <c r="J35" s="138">
+      <c r="J35" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>41.25</v>
       </c>
-      <c r="K35" s="138">
+      <c r="K35" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>24.75</v>
       </c>
-      <c r="L35" s="138">
+      <c r="L35" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>12.375</v>
       </c>
@@ -61455,19 +61449,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>12.75</v>
       </c>
-      <c r="I36" s="138">
+      <c r="I36" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>85</v>
       </c>
-      <c r="J36" s="138">
+      <c r="J36" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>42.5</v>
       </c>
-      <c r="K36" s="138">
+      <c r="K36" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>25.5</v>
       </c>
-      <c r="L36" s="138">
+      <c r="L36" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>12.75</v>
       </c>
@@ -61504,19 +61498,19 @@
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>13.125</v>
       </c>
-      <c r="I37" s="138">
+      <c r="I37" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_1*years_per_round</f>
         <v>87.5</v>
       </c>
-      <c r="J37" s="138">
+      <c r="J37" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_2*years_per_round</f>
         <v>43.75</v>
       </c>
-      <c r="K37" s="138">
+      <c r="K37" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_3*years_per_round</f>
         <v>26.25</v>
       </c>
-      <c r="L37" s="138">
+      <c r="L37" s="137">
         <f>Table8[[#This Row],[Netzbezug Real]]*real_zu_spiel_emissionsintensität_4*years_per_round</f>
         <v>13.125</v>
       </c>

</xml_diff>